<commit_message>
COBRANZA - NIVEL DE TIEMPO
</commit_message>
<xml_diff>
--- a/FabricaHilos/Data/CreditoCobranza/17. Creditos y Cobranzas - (GC) Nivel de morosidad 2026.xlsx
+++ b/FabricaHilos/Data/CreditoCobranza/17. Creditos y Cobranzas - (GC) Nivel de morosidad 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP710_03\LA COLONIAL Dropbox\Control Calidad La Colonial\SGC LA COLONIAL FABRICA DE HILOS\00. PROPUESTA\1. ISO 9001\4. Indicadores\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.Net\Dev\FabricaHilosRepository\FabricaHilos\Data\CreditoCobranza\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D210C5-0D15-44B2-87CF-8E3D4228DAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E5039A2-14A8-4F60-A7BC-B8ED25921467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="767" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -173,28 +173,6 @@
 </comments>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
@@ -223,9 +201,6 @@
   </si>
   <si>
     <t>FRECUENCIA DE SEGUIMIENTO Y MEDICIÓN</t>
-  </si>
-  <si>
-    <t>REPORTE DE INDICADOR DE DESEMPEÑO</t>
   </si>
   <si>
     <t>Promedio Anual</t>
@@ -380,6 +355,9 @@
   </si>
   <si>
     <t>Mariela Alvildo</t>
+  </si>
+  <si>
+    <t>REPORTE DE INDICADOR DE NIVEL MOROSIDAD</t>
   </si>
 </sst>
 </file>
@@ -1034,6 +1012,171 @@
     <xf numFmtId="9" fontId="41" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="39" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="39" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="37" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="35" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="37" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="32" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="37" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1126,171 +1269,6 @@
     </xf>
     <xf numFmtId="0" fontId="25" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="37" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="32" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="37" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="35" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="37" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2239,64 +2217,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
 <file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
 <richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <rel r:id="rId1"/>
@@ -2640,28 +2560,26 @@
     </row>
     <row r="2" spans="1:31" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="113" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C2" s="114"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="104" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="104"/>
-      <c r="I2" s="104"/>
-      <c r="J2" s="104"/>
-      <c r="K2" s="104"/>
-      <c r="L2" s="104"/>
-      <c r="M2" s="104"/>
-      <c r="N2" s="105" t="s">
-        <v>24</v>
-      </c>
-      <c r="O2" s="105"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="73" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="74" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="74"/>
       <c r="P2" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
@@ -2681,24 +2599,24 @@
     </row>
     <row r="3" spans="1:31" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="116"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="118"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104"/>
-      <c r="K3" s="104"/>
-      <c r="L3" s="104"/>
-      <c r="M3" s="104"/>
-      <c r="N3" s="111" t="s">
+      <c r="B3" s="85"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="73"/>
+      <c r="N3" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="81"/>
+      <c r="P3" s="14" t="s">
         <v>25</v>
-      </c>
-      <c r="O3" s="112"/>
-      <c r="P3" s="14" t="s">
-        <v>26</v>
       </c>
       <c r="Q3" s="2"/>
       <c r="R3" s="11"/>
@@ -2718,22 +2636,22 @@
     </row>
     <row r="4" spans="1:31" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="116"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="118"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="104"/>
-      <c r="H4" s="104"/>
-      <c r="I4" s="104"/>
-      <c r="J4" s="104"/>
-      <c r="K4" s="104"/>
-      <c r="L4" s="104"/>
-      <c r="M4" s="104"/>
-      <c r="N4" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="112"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="80" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4" s="81"/>
       <c r="P4" s="15">
         <v>46079</v>
       </c>
@@ -2755,24 +2673,24 @@
     </row>
     <row r="5" spans="1:31" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="104"/>
-      <c r="F5" s="104"/>
-      <c r="G5" s="104"/>
-      <c r="H5" s="104"/>
-      <c r="I5" s="104"/>
-      <c r="J5" s="104"/>
-      <c r="K5" s="104"/>
-      <c r="L5" s="104"/>
-      <c r="M5" s="104"/>
-      <c r="N5" s="111" t="s">
+      <c r="B5" s="85"/>
+      <c r="C5" s="86"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
+      <c r="L5" s="73"/>
+      <c r="M5" s="73"/>
+      <c r="N5" s="80" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="81"/>
+      <c r="P5" s="14" t="s">
         <v>30</v>
-      </c>
-      <c r="O5" s="112"/>
-      <c r="P5" s="14" t="s">
-        <v>31</v>
       </c>
       <c r="Q5" s="2"/>
       <c r="R5" s="11"/>
@@ -2792,24 +2710,24 @@
     </row>
     <row r="6" spans="1:31" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="119"/>
-      <c r="C6" s="120"/>
-      <c r="D6" s="121"/>
-      <c r="E6" s="104"/>
-      <c r="F6" s="104"/>
-      <c r="G6" s="104"/>
-      <c r="H6" s="104"/>
-      <c r="I6" s="104"/>
-      <c r="J6" s="104"/>
-      <c r="K6" s="104"/>
-      <c r="L6" s="104"/>
-      <c r="M6" s="104"/>
-      <c r="N6" s="111" t="s">
+      <c r="B6" s="88"/>
+      <c r="C6" s="89"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
+      <c r="L6" s="73"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="80" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="81"/>
+      <c r="P6" s="14" t="s">
         <v>28</v>
-      </c>
-      <c r="O6" s="112"/>
-      <c r="P6" s="14" t="s">
-        <v>29</v>
       </c>
       <c r="Q6" s="2"/>
       <c r="R6" s="11"/>
@@ -2862,29 +2780,29 @@
     </row>
     <row r="8" spans="1:31" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
-      <c r="B8" s="106" t="s">
+      <c r="B8" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="107"/>
-      <c r="D8" s="108"/>
-      <c r="E8" s="109" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="109"/>
-      <c r="G8" s="109"/>
-      <c r="H8" s="109"/>
-      <c r="I8" s="109"/>
-      <c r="J8" s="109"/>
-      <c r="K8" s="109"/>
-      <c r="L8" s="109"/>
-      <c r="M8" s="90" t="s">
+      <c r="C8" s="76"/>
+      <c r="D8" s="77"/>
+      <c r="E8" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="78"/>
+      <c r="K8" s="78"/>
+      <c r="L8" s="78"/>
+      <c r="M8" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="N8" s="90"/>
-      <c r="O8" s="110">
+      <c r="N8" s="72"/>
+      <c r="O8" s="79">
         <v>46023</v>
       </c>
-      <c r="P8" s="110"/>
+      <c r="P8" s="79"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="11"/>
       <c r="S8" s="11"/>
@@ -2936,29 +2854,29 @@
     </row>
     <row r="10" spans="1:31" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="87"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="89" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="89"/>
-      <c r="G10" s="89"/>
-      <c r="H10" s="89"/>
-      <c r="I10" s="89"/>
-      <c r="J10" s="89"/>
-      <c r="K10" s="89"/>
-      <c r="L10" s="89"/>
-      <c r="M10" s="90" t="s">
-        <v>46</v>
-      </c>
-      <c r="N10" s="90"/>
-      <c r="O10" s="91">
+      <c r="C10" s="92"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="94" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="94"/>
+      <c r="G10" s="94"/>
+      <c r="H10" s="94"/>
+      <c r="I10" s="94"/>
+      <c r="J10" s="94"/>
+      <c r="K10" s="94"/>
+      <c r="L10" s="94"/>
+      <c r="M10" s="72" t="s">
+        <v>45</v>
+      </c>
+      <c r="N10" s="72"/>
+      <c r="O10" s="95">
         <v>46357</v>
       </c>
-      <c r="P10" s="91"/>
+      <c r="P10" s="95"/>
       <c r="Q10" s="2"/>
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
@@ -3008,35 +2926,35 @@
     </row>
     <row r="12" spans="1:31" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
-      <c r="B12" s="125" t="s">
+      <c r="B12" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="125"/>
-      <c r="D12" s="125"/>
-      <c r="E12" s="99" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="99"/>
-      <c r="G12" s="99"/>
-      <c r="H12" s="99"/>
-      <c r="I12" s="90" t="s">
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="71" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="71"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="71"/>
+      <c r="I12" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="J12" s="90"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L12" s="50">
         <v>0.1</v>
       </c>
-      <c r="M12" s="90" t="s">
+      <c r="M12" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="N12" s="90"/>
-      <c r="O12" s="99" t="s">
-        <v>45</v>
-      </c>
-      <c r="P12" s="99"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="71" t="s">
+        <v>44</v>
+      </c>
+      <c r="P12" s="71"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="11"/>
       <c r="S12" s="11"/>
@@ -3086,27 +3004,27 @@
     </row>
     <row r="14" spans="1:31" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
-      <c r="B14" s="100" t="s">
+      <c r="B14" s="103" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="103"/>
+      <c r="D14" s="103"/>
+      <c r="E14" s="104" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="105"/>
+      <c r="G14" s="105"/>
+      <c r="H14" s="106"/>
+      <c r="I14" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="100"/>
-      <c r="D14" s="100"/>
-      <c r="E14" s="101" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="102"/>
-      <c r="G14" s="102"/>
-      <c r="H14" s="103"/>
-      <c r="I14" s="86" t="s">
-        <v>13</v>
-      </c>
-      <c r="J14" s="88"/>
-      <c r="K14" s="122"/>
-      <c r="L14" s="123"/>
-      <c r="M14" s="123"/>
-      <c r="N14" s="123"/>
-      <c r="O14" s="123"/>
-      <c r="P14" s="124"/>
+      <c r="J14" s="93"/>
+      <c r="K14" s="67"/>
+      <c r="L14" s="68"/>
+      <c r="M14" s="68"/>
+      <c r="N14" s="68"/>
+      <c r="O14" s="68"/>
+      <c r="P14" s="69"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="11"/>
       <c r="S14" s="11"/>
@@ -3157,33 +3075,33 @@
       <c r="AE15" s="11"/>
     </row>
     <row r="16" spans="1:31" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="94" t="s">
+      <c r="B16" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="94"/>
-      <c r="D16" s="94"/>
-      <c r="E16" s="131" t="s">
-        <v>49</v>
-      </c>
-      <c r="F16" s="132"/>
+      <c r="C16" s="98"/>
+      <c r="D16" s="98"/>
+      <c r="E16" s="52" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="53"/>
       <c r="G16" s="43">
         <f>L12</f>
         <v>0.1</v>
       </c>
       <c r="H16" s="44"/>
       <c r="I16" s="45"/>
-      <c r="J16" s="95"/>
-      <c r="K16" s="96"/>
+      <c r="J16" s="99"/>
+      <c r="K16" s="100"/>
       <c r="L16" s="46"/>
       <c r="M16" s="47"/>
       <c r="N16" s="48">
         <f>L12</f>
         <v>0.1</v>
       </c>
-      <c r="O16" s="133" t="s">
-        <v>50</v>
-      </c>
-      <c r="P16" s="134"/>
+      <c r="O16" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="P16" s="55"/>
       <c r="R16" s="49"/>
       <c r="S16" s="49"/>
       <c r="T16" s="49"/>
@@ -3234,23 +3152,23 @@
     </row>
     <row r="18" spans="1:31" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
-      <c r="B18" s="97" t="s">
+      <c r="B18" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="97"/>
-      <c r="D18" s="97"/>
-      <c r="E18" s="97"/>
-      <c r="F18" s="97"/>
-      <c r="G18" s="97"/>
-      <c r="H18" s="97"/>
-      <c r="I18" s="97"/>
-      <c r="J18" s="97"/>
-      <c r="K18" s="97"/>
-      <c r="L18" s="97"/>
-      <c r="M18" s="97"/>
-      <c r="N18" s="97"/>
-      <c r="O18" s="97"/>
-      <c r="P18" s="97"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="101"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="101"/>
+      <c r="J18" s="101"/>
+      <c r="K18" s="101"/>
+      <c r="L18" s="101"/>
+      <c r="M18" s="101"/>
+      <c r="N18" s="101"/>
+      <c r="O18" s="101"/>
+      <c r="P18" s="101"/>
       <c r="Q18" s="2"/>
       <c r="R18" s="11"/>
       <c r="S18" s="11"/>
@@ -3269,9 +3187,9 @@
     </row>
     <row r="19" spans="1:31" s="1" customFormat="1" ht="299.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="98"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="98"/>
+      <c r="B19" s="102"/>
+      <c r="C19" s="102"/>
+      <c r="D19" s="102"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="2"/>
@@ -3336,52 +3254,52 @@
     <row r="21" spans="1:31" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="D21" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="F21" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="G21" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="H21" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="I21" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="I21" s="17" t="s">
+      <c r="J21" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="J21" s="17" t="s">
+      <c r="K21" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="K21" s="17" t="s">
+      <c r="L21" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="L21" s="17" t="s">
+      <c r="M21" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="M21" s="17" t="s">
+      <c r="N21" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="N21" s="17" t="s">
+      <c r="O21" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="O21" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="P21" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:31" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="B22" s="92" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="93"/>
+      <c r="B22" s="96" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="97"/>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
@@ -3402,10 +3320,10 @@
     </row>
     <row r="23" spans="1:31" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="B23" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="93"/>
+      <c r="B23" s="96" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="97"/>
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
       <c r="F23" s="19"/>
@@ -3426,10 +3344,10 @@
     </row>
     <row r="24" spans="1:31" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="92" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" s="93"/>
+      <c r="B24" s="96" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="97"/>
       <c r="D24" s="24" t="str">
         <f>IFERROR(D22/D23,"")</f>
         <v/>
@@ -3486,10 +3404,10 @@
     </row>
     <row r="25" spans="1:31" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
-      <c r="B25" s="92" t="s">
+      <c r="B25" s="96" t="s">
         <v>3</v>
       </c>
-      <c r="C25" s="93"/>
+      <c r="C25" s="97"/>
       <c r="D25" s="25">
         <f>$L$12</f>
         <v>0.1</v>
@@ -3546,25 +3464,25 @@
     </row>
     <row r="26" spans="1:31" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
-      <c r="B26" s="53" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56" t="s">
-        <v>21</v>
-      </c>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="57"/>
-      <c r="L26" s="57"/>
-      <c r="M26" s="57"/>
-      <c r="N26" s="57"/>
-      <c r="O26" s="57"/>
-      <c r="P26" s="58"/>
+      <c r="B26" s="108" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="110"/>
+      <c r="G26" s="111" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" s="112"/>
+      <c r="I26" s="112"/>
+      <c r="J26" s="112"/>
+      <c r="K26" s="112"/>
+      <c r="L26" s="112"/>
+      <c r="M26" s="112"/>
+      <c r="N26" s="112"/>
+      <c r="O26" s="112"/>
+      <c r="P26" s="113"/>
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:31" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3588,282 +3506,282 @@
     </row>
     <row r="28" spans="1:31" s="3" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
-      <c r="B28" s="59" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="60"/>
-      <c r="J28" s="60"/>
-      <c r="K28" s="60"/>
-      <c r="L28" s="60"/>
-      <c r="M28" s="60"/>
-      <c r="N28" s="60"/>
-      <c r="O28" s="60"/>
-      <c r="P28" s="61"/>
+      <c r="B28" s="114" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="115"/>
+      <c r="D28" s="115"/>
+      <c r="E28" s="115"/>
+      <c r="F28" s="115"/>
+      <c r="G28" s="115"/>
+      <c r="H28" s="115"/>
+      <c r="I28" s="115"/>
+      <c r="J28" s="115"/>
+      <c r="K28" s="115"/>
+      <c r="L28" s="115"/>
+      <c r="M28" s="115"/>
+      <c r="N28" s="115"/>
+      <c r="O28" s="115"/>
+      <c r="P28" s="116"/>
       <c r="Q28" s="4"/>
     </row>
     <row r="29" spans="1:31" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
-      <c r="B29" s="63" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="64"/>
-      <c r="D29" s="64"/>
-      <c r="E29" s="64"/>
-      <c r="F29" s="64"/>
-      <c r="G29" s="65"/>
-      <c r="H29" s="72"/>
-      <c r="I29" s="72"/>
-      <c r="J29" s="72"/>
-      <c r="K29" s="72"/>
-      <c r="L29" s="72"/>
-      <c r="M29" s="72"/>
-      <c r="N29" s="72"/>
-      <c r="O29" s="72"/>
-      <c r="P29" s="73"/>
+      <c r="B29" s="118" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="119"/>
+      <c r="D29" s="119"/>
+      <c r="E29" s="119"/>
+      <c r="F29" s="119"/>
+      <c r="G29" s="120"/>
+      <c r="H29" s="127"/>
+      <c r="I29" s="127"/>
+      <c r="J29" s="127"/>
+      <c r="K29" s="127"/>
+      <c r="L29" s="127"/>
+      <c r="M29" s="127"/>
+      <c r="N29" s="127"/>
+      <c r="O29" s="127"/>
+      <c r="P29" s="128"/>
       <c r="Q29" s="4"/>
     </row>
     <row r="30" spans="1:31" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
-      <c r="B30" s="66"/>
-      <c r="C30" s="67"/>
-      <c r="D30" s="67"/>
-      <c r="E30" s="67"/>
-      <c r="F30" s="67"/>
-      <c r="G30" s="68"/>
-      <c r="H30" s="74"/>
-      <c r="I30" s="74"/>
-      <c r="J30" s="74"/>
-      <c r="K30" s="74"/>
-      <c r="L30" s="74"/>
-      <c r="M30" s="74"/>
-      <c r="N30" s="74"/>
-      <c r="O30" s="74"/>
-      <c r="P30" s="75"/>
+      <c r="B30" s="121"/>
+      <c r="C30" s="122"/>
+      <c r="D30" s="122"/>
+      <c r="E30" s="122"/>
+      <c r="F30" s="122"/>
+      <c r="G30" s="123"/>
+      <c r="H30" s="129"/>
+      <c r="I30" s="129"/>
+      <c r="J30" s="129"/>
+      <c r="K30" s="129"/>
+      <c r="L30" s="129"/>
+      <c r="M30" s="129"/>
+      <c r="N30" s="129"/>
+      <c r="O30" s="129"/>
+      <c r="P30" s="130"/>
       <c r="Q30" s="4"/>
     </row>
     <row r="31" spans="1:31" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
-      <c r="B31" s="66"/>
-      <c r="C31" s="67"/>
-      <c r="D31" s="67"/>
-      <c r="E31" s="67"/>
-      <c r="F31" s="67"/>
-      <c r="G31" s="68"/>
-      <c r="H31" s="74"/>
-      <c r="I31" s="74"/>
-      <c r="J31" s="74"/>
-      <c r="K31" s="74"/>
-      <c r="L31" s="74"/>
-      <c r="M31" s="74"/>
-      <c r="N31" s="74"/>
-      <c r="O31" s="74"/>
-      <c r="P31" s="75"/>
+      <c r="B31" s="121"/>
+      <c r="C31" s="122"/>
+      <c r="D31" s="122"/>
+      <c r="E31" s="122"/>
+      <c r="F31" s="122"/>
+      <c r="G31" s="123"/>
+      <c r="H31" s="129"/>
+      <c r="I31" s="129"/>
+      <c r="J31" s="129"/>
+      <c r="K31" s="129"/>
+      <c r="L31" s="129"/>
+      <c r="M31" s="129"/>
+      <c r="N31" s="129"/>
+      <c r="O31" s="129"/>
+      <c r="P31" s="130"/>
       <c r="Q31" s="4"/>
     </row>
     <row r="32" spans="1:31" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
-      <c r="B32" s="66"/>
-      <c r="C32" s="67"/>
-      <c r="D32" s="67"/>
-      <c r="E32" s="67"/>
-      <c r="F32" s="67"/>
-      <c r="G32" s="68"/>
-      <c r="H32" s="74"/>
-      <c r="I32" s="74"/>
-      <c r="J32" s="74"/>
-      <c r="K32" s="74"/>
-      <c r="L32" s="74"/>
-      <c r="M32" s="74"/>
-      <c r="N32" s="74"/>
-      <c r="O32" s="74"/>
-      <c r="P32" s="75"/>
+      <c r="B32" s="121"/>
+      <c r="C32" s="122"/>
+      <c r="D32" s="122"/>
+      <c r="E32" s="122"/>
+      <c r="F32" s="122"/>
+      <c r="G32" s="123"/>
+      <c r="H32" s="129"/>
+      <c r="I32" s="129"/>
+      <c r="J32" s="129"/>
+      <c r="K32" s="129"/>
+      <c r="L32" s="129"/>
+      <c r="M32" s="129"/>
+      <c r="N32" s="129"/>
+      <c r="O32" s="129"/>
+      <c r="P32" s="130"/>
       <c r="Q32" s="4"/>
     </row>
     <row r="33" spans="1:17" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
-      <c r="B33" s="66"/>
-      <c r="C33" s="67"/>
-      <c r="D33" s="67"/>
-      <c r="E33" s="67"/>
-      <c r="F33" s="67"/>
-      <c r="G33" s="68"/>
-      <c r="H33" s="74"/>
-      <c r="I33" s="74"/>
-      <c r="J33" s="74"/>
-      <c r="K33" s="74"/>
-      <c r="L33" s="74"/>
-      <c r="M33" s="74"/>
-      <c r="N33" s="74"/>
-      <c r="O33" s="74"/>
-      <c r="P33" s="75"/>
+      <c r="B33" s="121"/>
+      <c r="C33" s="122"/>
+      <c r="D33" s="122"/>
+      <c r="E33" s="122"/>
+      <c r="F33" s="122"/>
+      <c r="G33" s="123"/>
+      <c r="H33" s="129"/>
+      <c r="I33" s="129"/>
+      <c r="J33" s="129"/>
+      <c r="K33" s="129"/>
+      <c r="L33" s="129"/>
+      <c r="M33" s="129"/>
+      <c r="N33" s="129"/>
+      <c r="O33" s="129"/>
+      <c r="P33" s="130"/>
       <c r="Q33" s="4"/>
     </row>
     <row r="34" spans="1:17" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="69"/>
-      <c r="C34" s="70"/>
-      <c r="D34" s="70"/>
-      <c r="E34" s="70"/>
-      <c r="F34" s="70"/>
-      <c r="G34" s="71"/>
-      <c r="H34" s="76"/>
-      <c r="I34" s="77"/>
-      <c r="J34" s="77"/>
-      <c r="K34" s="77"/>
-      <c r="L34" s="77"/>
-      <c r="M34" s="77"/>
-      <c r="N34" s="77"/>
-      <c r="O34" s="77"/>
-      <c r="P34" s="78"/>
+      <c r="B34" s="124"/>
+      <c r="C34" s="125"/>
+      <c r="D34" s="125"/>
+      <c r="E34" s="125"/>
+      <c r="F34" s="125"/>
+      <c r="G34" s="126"/>
+      <c r="H34" s="131"/>
+      <c r="I34" s="132"/>
+      <c r="J34" s="132"/>
+      <c r="K34" s="132"/>
+      <c r="L34" s="132"/>
+      <c r="M34" s="132"/>
+      <c r="N34" s="132"/>
+      <c r="O34" s="132"/>
+      <c r="P34" s="133"/>
       <c r="Q34" s="4"/>
     </row>
     <row r="35" spans="1:17" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="79"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="79"/>
-      <c r="E35" s="79"/>
-      <c r="F35" s="79"/>
-      <c r="G35" s="79"/>
-      <c r="H35" s="79"/>
-      <c r="I35" s="79"/>
-      <c r="J35" s="79"/>
-      <c r="K35" s="79"/>
-      <c r="L35" s="79"/>
-      <c r="M35" s="79"/>
-      <c r="N35" s="79"/>
-      <c r="O35" s="79"/>
-      <c r="P35" s="79"/>
+      <c r="B35" s="134"/>
+      <c r="C35" s="134"/>
+      <c r="D35" s="134"/>
+      <c r="E35" s="134"/>
+      <c r="F35" s="134"/>
+      <c r="G35" s="134"/>
+      <c r="H35" s="134"/>
+      <c r="I35" s="134"/>
+      <c r="J35" s="134"/>
+      <c r="K35" s="134"/>
+      <c r="L35" s="134"/>
+      <c r="M35" s="134"/>
+      <c r="N35" s="134"/>
+      <c r="O35" s="134"/>
+      <c r="P35" s="134"/>
       <c r="Q35" s="4"/>
     </row>
     <row r="36" spans="1:17" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="59" t="s">
-        <v>16</v>
-      </c>
-      <c r="C36" s="60"/>
-      <c r="D36" s="60"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="60"/>
-      <c r="G36" s="60"/>
-      <c r="H36" s="60"/>
-      <c r="I36" s="60"/>
-      <c r="J36" s="60"/>
-      <c r="K36" s="60"/>
-      <c r="L36" s="60"/>
-      <c r="M36" s="60"/>
-      <c r="N36" s="60"/>
-      <c r="O36" s="60"/>
-      <c r="P36" s="61"/>
+      <c r="B36" s="114" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="115"/>
+      <c r="D36" s="115"/>
+      <c r="E36" s="115"/>
+      <c r="F36" s="115"/>
+      <c r="G36" s="115"/>
+      <c r="H36" s="115"/>
+      <c r="I36" s="115"/>
+      <c r="J36" s="115"/>
+      <c r="K36" s="115"/>
+      <c r="L36" s="115"/>
+      <c r="M36" s="115"/>
+      <c r="N36" s="115"/>
+      <c r="O36" s="115"/>
+      <c r="P36" s="116"/>
       <c r="Q36" s="4"/>
     </row>
     <row r="37" spans="1:17" s="3" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
-      <c r="B37" s="80"/>
-      <c r="C37" s="81"/>
-      <c r="D37" s="81"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="81"/>
-      <c r="G37" s="81"/>
-      <c r="H37" s="81"/>
-      <c r="I37" s="81"/>
-      <c r="J37" s="81"/>
-      <c r="K37" s="81"/>
-      <c r="L37" s="81"/>
-      <c r="M37" s="81"/>
-      <c r="N37" s="81"/>
-      <c r="O37" s="81"/>
-      <c r="P37" s="82"/>
+      <c r="B37" s="135"/>
+      <c r="C37" s="136"/>
+      <c r="D37" s="136"/>
+      <c r="E37" s="136"/>
+      <c r="F37" s="136"/>
+      <c r="G37" s="136"/>
+      <c r="H37" s="136"/>
+      <c r="I37" s="136"/>
+      <c r="J37" s="136"/>
+      <c r="K37" s="136"/>
+      <c r="L37" s="136"/>
+      <c r="M37" s="136"/>
+      <c r="N37" s="136"/>
+      <c r="O37" s="136"/>
+      <c r="P37" s="137"/>
       <c r="Q37" s="4"/>
     </row>
     <row r="38" spans="1:17" s="3" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
-      <c r="B38" s="135" t="s">
+      <c r="B38" s="56" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="57"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="57"/>
+      <c r="F38" s="57"/>
+      <c r="G38" s="57"/>
+      <c r="H38" s="58"/>
+      <c r="I38" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="C38" s="136"/>
-      <c r="D38" s="136"/>
-      <c r="E38" s="136"/>
-      <c r="F38" s="136"/>
-      <c r="G38" s="136"/>
-      <c r="H38" s="137"/>
-      <c r="I38" s="135" t="s">
+      <c r="J38" s="57"/>
+      <c r="K38" s="58"/>
+      <c r="L38" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="J38" s="136"/>
-      <c r="K38" s="137"/>
-      <c r="L38" s="135" t="s">
+      <c r="M38" s="58"/>
+      <c r="N38" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="137"/>
-      <c r="N38" s="135" t="s">
-        <v>20</v>
-      </c>
-      <c r="O38" s="136"/>
-      <c r="P38" s="137"/>
+      <c r="O38" s="57"/>
+      <c r="P38" s="58"/>
       <c r="Q38" s="4"/>
     </row>
     <row r="39" spans="1:17" s="3" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
-      <c r="B39" s="83"/>
-      <c r="C39" s="84"/>
-      <c r="D39" s="84"/>
-      <c r="E39" s="84"/>
-      <c r="F39" s="84"/>
-      <c r="G39" s="84"/>
-      <c r="H39" s="85"/>
-      <c r="I39" s="83"/>
-      <c r="J39" s="84"/>
-      <c r="K39" s="85"/>
-      <c r="L39" s="126"/>
-      <c r="M39" s="127"/>
-      <c r="N39" s="128"/>
-      <c r="O39" s="129"/>
-      <c r="P39" s="130"/>
+      <c r="B39" s="59"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="60"/>
+      <c r="E39" s="60"/>
+      <c r="F39" s="60"/>
+      <c r="G39" s="60"/>
+      <c r="H39" s="61"/>
+      <c r="I39" s="59"/>
+      <c r="J39" s="60"/>
+      <c r="K39" s="61"/>
+      <c r="L39" s="62"/>
+      <c r="M39" s="63"/>
+      <c r="N39" s="64"/>
+      <c r="O39" s="65"/>
+      <c r="P39" s="66"/>
       <c r="Q39" s="4"/>
     </row>
     <row r="40" spans="1:17" s="3" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
-      <c r="B40" s="83"/>
-      <c r="C40" s="84"/>
-      <c r="D40" s="84"/>
-      <c r="E40" s="84"/>
-      <c r="F40" s="84"/>
-      <c r="G40" s="84"/>
-      <c r="H40" s="85"/>
-      <c r="I40" s="83"/>
-      <c r="J40" s="84"/>
-      <c r="K40" s="85"/>
-      <c r="L40" s="126"/>
-      <c r="M40" s="127"/>
-      <c r="N40" s="128"/>
-      <c r="O40" s="129"/>
-      <c r="P40" s="130"/>
+      <c r="B40" s="59"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="60"/>
+      <c r="E40" s="60"/>
+      <c r="F40" s="60"/>
+      <c r="G40" s="60"/>
+      <c r="H40" s="61"/>
+      <c r="I40" s="59"/>
+      <c r="J40" s="60"/>
+      <c r="K40" s="61"/>
+      <c r="L40" s="62"/>
+      <c r="M40" s="63"/>
+      <c r="N40" s="64"/>
+      <c r="O40" s="65"/>
+      <c r="P40" s="66"/>
       <c r="Q40" s="4"/>
     </row>
     <row r="41" spans="1:17" s="3" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
-      <c r="B41" s="83"/>
-      <c r="C41" s="84"/>
-      <c r="D41" s="84"/>
-      <c r="E41" s="84"/>
-      <c r="F41" s="84"/>
-      <c r="G41" s="84"/>
-      <c r="H41" s="85"/>
-      <c r="I41" s="83"/>
-      <c r="J41" s="84"/>
-      <c r="K41" s="85"/>
-      <c r="L41" s="126"/>
-      <c r="M41" s="127"/>
-      <c r="N41" s="128"/>
-      <c r="O41" s="129"/>
-      <c r="P41" s="130"/>
+      <c r="B41" s="59"/>
+      <c r="C41" s="60"/>
+      <c r="D41" s="60"/>
+      <c r="E41" s="60"/>
+      <c r="F41" s="60"/>
+      <c r="G41" s="60"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="59"/>
+      <c r="J41" s="60"/>
+      <c r="K41" s="61"/>
+      <c r="L41" s="62"/>
+      <c r="M41" s="63"/>
+      <c r="N41" s="64"/>
+      <c r="O41" s="65"/>
+      <c r="P41" s="66"/>
       <c r="Q41" s="4"/>
     </row>
     <row r="42" spans="1:17" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3916,11 +3834,11 @@
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
       <c r="K44" s="4"/>
-      <c r="L44" s="62" t="s">
-        <v>56</v>
-      </c>
-      <c r="M44" s="62"/>
-      <c r="N44" s="62"/>
+      <c r="L44" s="117" t="s">
+        <v>55</v>
+      </c>
+      <c r="M44" s="117"/>
+      <c r="N44" s="117"/>
       <c r="O44" s="4"/>
       <c r="P44" s="4"/>
     </row>
@@ -3936,11 +3854,11 @@
       <c r="I45" s="4"/>
       <c r="J45" s="4"/>
       <c r="K45" s="4"/>
-      <c r="L45" s="52" t="s">
-        <v>55</v>
-      </c>
-      <c r="M45" s="52"/>
-      <c r="N45" s="52"/>
+      <c r="L45" s="107" t="s">
+        <v>54</v>
+      </c>
+      <c r="M45" s="107"/>
+      <c r="N45" s="107"/>
       <c r="O45" s="4"/>
       <c r="P45" s="4"/>
     </row>
@@ -3951,39 +3869,22 @@
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="N38:P38"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="N41:P41"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="N39:P39"/>
-    <mergeCell ref="B40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="N40:P40"/>
-    <mergeCell ref="K14:P14"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="E12:H12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="E2:M6"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="E8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="B2:D6"/>
+    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="G26:P26"/>
+    <mergeCell ref="B28:P28"/>
+    <mergeCell ref="L44:N44"/>
+    <mergeCell ref="B29:G34"/>
+    <mergeCell ref="H29:P29"/>
+    <mergeCell ref="H30:P30"/>
+    <mergeCell ref="H31:P31"/>
+    <mergeCell ref="H32:P32"/>
+    <mergeCell ref="H33:P33"/>
+    <mergeCell ref="H34:P34"/>
+    <mergeCell ref="B35:P35"/>
+    <mergeCell ref="B36:P36"/>
+    <mergeCell ref="B37:P37"/>
+    <mergeCell ref="B41:H41"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="E10:L10"/>
     <mergeCell ref="M10:N10"/>
@@ -4000,22 +3901,39 @@
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:H14"/>
     <mergeCell ref="I14:J14"/>
-    <mergeCell ref="L45:N45"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="G26:P26"/>
-    <mergeCell ref="B28:P28"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="B29:G34"/>
-    <mergeCell ref="H29:P29"/>
-    <mergeCell ref="H30:P30"/>
-    <mergeCell ref="H31:P31"/>
-    <mergeCell ref="H32:P32"/>
-    <mergeCell ref="H33:P33"/>
-    <mergeCell ref="H34:P34"/>
-    <mergeCell ref="B35:P35"/>
-    <mergeCell ref="B36:P36"/>
-    <mergeCell ref="B37:P37"/>
-    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="E2:M6"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="E8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="B2:D6"/>
+    <mergeCell ref="K14:P14"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="N41:P41"/>
+    <mergeCell ref="B39:H39"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="N39:P39"/>
+    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="N40:P40"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="B38:H38"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="N38:P38"/>
   </mergeCells>
   <conditionalFormatting sqref="D24:P24">
     <cfRule type="cellIs" dxfId="3" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>